<commit_message>
AB-engine layout tree and lengths from Route 16 (Rev J); Route 3/4 engine tree deleted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -651,7 +651,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2470</t>
+          <t>1342</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>920</t>
+          <t>1088</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>740</t>
+          <t>1005</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>560</t>
+          <t>900</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>795</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1180</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>1023</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>1023</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1190</t>
+          <t>852</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>765</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>684</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>619</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>610</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>610</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1380</t>
+          <t>1158</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>980</t>
+          <t>1158</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>982</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2615,7 +2615,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>982</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>700</t>
+          <t>1085</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3423,7 +3423,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3535,7 +3535,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3995,7 +3995,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>1030</t>
+          <t>953</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1060</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1110</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4779,7 +4779,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>1380</t>
+          <t>1175</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -5011,7 +5011,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1175</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>1450</t>
+          <t>925</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -5235,7 +5235,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>648</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>648</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5463,7 +5463,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>648</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1007</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1007</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5807,7 +5807,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1007</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>1580</t>
+          <t>1251</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>1580</t>
+          <t>1251</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>652</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -6363,7 +6363,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>652</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>652</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -6591,7 +6591,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>262</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>109</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>293</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>510</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>210</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>427</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -7843,7 +7843,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>105</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>322</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>217</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>234</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>136</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>291</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -8647,7 +8647,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>115</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -8767,7 +8767,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>410</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>394</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>275</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>188</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -9223,7 +9223,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>107</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -9339,7 +9339,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>42</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -9455,7 +9455,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>156</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>657</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -9679,7 +9679,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>484</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>1380</t>
+          <t>1175</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -10375,7 +10375,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -10499,7 +10499,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>715</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -10607,7 +10607,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>795</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -10723,7 +10723,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>501</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -10835,7 +10835,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>501</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
@@ -10943,7 +10943,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>691</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -11055,7 +11055,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>691</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>867</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -11279,7 +11279,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>577</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>691</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">

</xml_diff>

<commit_message>
AB-engine layout tree and lengths from Route 16 (Rev J); Route 3/4 engine tree deleted (#415)
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -651,7 +651,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2470</t>
+          <t>1342</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>920</t>
+          <t>1088</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>740</t>
+          <t>1005</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>560</t>
+          <t>900</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>795</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1180</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>1023</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>1023</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1190</t>
+          <t>852</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1020</t>
+          <t>765</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>684</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>619</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1820</t>
+          <t>610</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1420</t>
+          <t>610</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1380</t>
+          <t>1158</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>980</t>
+          <t>1158</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>530</t>
+          <t>982</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2615,7 +2615,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>982</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>700</t>
+          <t>1085</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>730</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3423,7 +3423,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3535,7 +3535,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>827</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3995,7 +3995,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1077</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>1030</t>
+          <t>953</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1060</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1110</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4779,7 +4779,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>618</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>1380</t>
+          <t>1175</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -5011,7 +5011,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1175</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>1450</t>
+          <t>925</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -5235,7 +5235,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>648</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>648</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5463,7 +5463,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>648</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1007</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>1007</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5807,7 +5807,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1007</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>1580</t>
+          <t>1251</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>1580</t>
+          <t>1251</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>652</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -6363,7 +6363,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>652</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>1460</t>
+          <t>652</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -6591,7 +6591,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>262</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1279</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>109</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>293</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>510</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>210</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>427</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -7843,7 +7843,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>105</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>322</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>217</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>234</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -8403,7 +8403,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>136</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>291</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -8647,7 +8647,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>115</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -8767,7 +8767,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>410</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>394</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>275</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>188</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -9223,7 +9223,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>107</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -9339,7 +9339,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>42</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -9455,7 +9455,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>156</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>657</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -9679,7 +9679,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>484</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>1380</t>
+          <t>1175</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -10375,7 +10375,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -10499,7 +10499,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>715</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -10607,7 +10607,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>795</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -10723,7 +10723,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>501</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -10835,7 +10835,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>501</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
@@ -10943,7 +10943,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>691</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -11055,7 +11055,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>691</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>867</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -11279,7 +11279,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>577</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>691</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">

</xml_diff>

<commit_message>
Coil ground straight to the POWER box NEG bar on bulkhead cavity 4 (Rev K)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -15,9 +15,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Wires'!$A$1:$Z$99</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Connectors'!$A$1:$I$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Connectors'!$A$1:$I$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Splices'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spare Cavities'!$A$1:$D$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spare Cavities'!$A$1:$D$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -6135,7 +6135,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>607</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>1279</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -7471,12 +7471,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ENG-GND-RING</t>
+          <t>DRB102-ENGINE</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -7511,7 +7511,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>293</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -7556,7 +7556,11 @@
           <t>SP-CHASSIS-ENG</t>
         </is>
       </c>
-      <c r="W63" t="inlineStr"/>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>ST185-AB-cabin w_cop_gnd_ac at DRB102-CABIN 4, to POWER-NEG-BAR Lug</t>
+        </is>
+      </c>
       <c r="X63" t="inlineStr"/>
       <c r="Y63" t="inlineStr"/>
       <c r="Z63" t="inlineStr"/>
@@ -7695,12 +7699,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>ENG-GND-RING</t>
+          <t>DRB102-ENGINE</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -7735,7 +7739,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>210</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -7780,7 +7784,11 @@
           <t>SP-CHASSIS-ENG</t>
         </is>
       </c>
-      <c r="W65" t="inlineStr"/>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>ST185-AB-cabin w_cop_gnd_ac at DRB102-CABIN 4, to POWER-NEG-BAR Lug</t>
+        </is>
+      </c>
       <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr"/>
       <c r="Z65" t="inlineStr"/>
@@ -7919,12 +7927,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ENG-GND-RING</t>
+          <t>DRB102-ENGINE</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -7959,7 +7967,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>105</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -8004,7 +8012,11 @@
           <t>SP-CHASSIS-ENG</t>
         </is>
       </c>
-      <c r="W67" t="inlineStr"/>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>ST185-AB-cabin w_cop_gnd_ac at DRB102-CABIN 4, to POWER-NEG-BAR Lug</t>
+        </is>
+      </c>
       <c r="X67" t="inlineStr"/>
       <c r="Y67" t="inlineStr"/>
       <c r="Z67" t="inlineStr"/>
@@ -8067,7 +8079,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>30</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -8143,12 +8155,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ENG-GND-RING</t>
+          <t>DRB102-ENGINE</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -8183,7 +8195,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>30</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -8228,7 +8240,11 @@
           <t>SP-CHASSIS-ENG</t>
         </is>
       </c>
-      <c r="W69" t="inlineStr"/>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>ST185-AB-cabin w_cop_gnd_ac at DRB102-CABIN 4, to POWER-NEG-BAR Lug</t>
+        </is>
+      </c>
       <c r="X69" t="inlineStr"/>
       <c r="Y69" t="inlineStr"/>
       <c r="Z69" t="inlineStr"/>
@@ -10444,7 +10460,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>w_eng_gnd</t>
+          <t>w_cop_gnd_e_ae</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -10459,12 +10475,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>ENG-GND-RING</t>
+          <t>DRB102-ENGINE</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10479,7 +10495,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Coil ground</t>
+          <t>Coil ground to the POWER box NEG bar</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -10489,22 +10505,22 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Blue-Yellow-Yellow</t>
+          <t>Blue-White-Yellow-Yellow</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>715</t>
+          <t>795</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>M22759/16-10-0</t>
+          <t>M22759/16-12-0</t>
         </is>
       </c>
       <c r="N89" t="inlineStr"/>
@@ -10516,22 +10532,22 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>0462-210-1231</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>Coil ground splice - ignition coils 1-4 to the engine block ground stud</t>
+          <t>Coil ground splice - ignition coils 1-4 to bulkhead pin 4 (POWER box NEG bar)</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>Engine block ground stud (RADLOK engine ground, H6), M6 ring</t>
+          <t>BULKHEAD</t>
         </is>
       </c>
       <c r="T89" t="inlineStr">
         <is>
-          <t>EGND</t>
+          <t>COPG</t>
         </is>
       </c>
       <c r="U89" t="inlineStr">
@@ -10544,10 +10560,18 @@
           <t>SP-CHASSIS-ENG</t>
         </is>
       </c>
-      <c r="W89" t="inlineStr"/>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>ST185-AB-cabin w_cop_gnd_ac at DRB102-CABIN 4, to POWER-NEG-BAR Lug</t>
+        </is>
+      </c>
       <c r="X89" t="inlineStr"/>
       <c r="Y89" t="inlineStr"/>
-      <c r="Z89" t="inlineStr"/>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>Dan 2026-10-29: coil ground straight to the glove-box POWER box NEG bar (cleanest return), not the engine block stud; 12 AWG like the COP feed (w_cop_pwr_e_ae, size-12 cavity 1); size-12 contact 12-14 AWG</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -11693,7 +11717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12180,10 +12204,10 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H12" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -12900,7 +12924,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ENG-GND-RING</t>
+          <t>STARTER-TRIGGER</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -12911,7 +12935,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Engine block ground stud (RADLOK engine ground, H6), M6 ring</t>
+          <t>Starter solenoid S (50) terminal post, spade</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -12931,28 +12955,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>STARTER-TRIGGER</t>
+          <t>SP-CANH-LAM</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>terminal</t>
+          <t>splice</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Starter solenoid S (50) terminal post, spade</t>
+          <t>CAN H join - bulkhead, Lambda, 120 ohm end</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>solder splice</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -12962,7 +12986,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SP-CANH-LAM</t>
+          <t>SP-CANL-LAM</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -12973,7 +12997,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CAN H join - bulkhead, Lambda, 120 ohm end</t>
+          <t>CAN L join - bulkhead, Lambda, 120 ohm end</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -12993,7 +13017,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SP-CANL-LAM</t>
+          <t>SP-CHASSIS-ENG</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -13004,7 +13028,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CAN L join - bulkhead, Lambda, 120 ohm end</t>
+          <t>Coil ground splice - ignition coils 1-4 to bulkhead pin 4 (POWER box NEG bar)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -13014,7 +13038,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -13024,7 +13048,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SP-CHASSIS-ENG</t>
+          <t>SP-COP-ENG</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -13035,7 +13059,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Coil ground splice - ignition coils 1-4 to the engine block ground stud</t>
+          <t>Coil +12 V splice - BH-A pin 1 (LOGIC COP 15A) to coils 1-4</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -13055,7 +13079,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SP-COP-ENG</t>
+          <t>SP-GNDOUT-B-ENG</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -13066,7 +13090,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Coil +12 V splice - BH-A pin 1 (LOGIC COP 15A) to coils 1-4</t>
+          <t>Sensor return splice - oil temp and charge temp, tied to the BH-B pin 29 splice</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -13076,7 +13100,7 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -13086,7 +13110,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SP-GNDOUT-B-ENG</t>
+          <t>SP-GNDOUT-B-ENG2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -13097,7 +13121,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Sensor return splice - oil temp and charge temp, tied to the BH-B pin 29 splice</t>
+          <t>Sensor return splice - BH-B pin 29 (ECU B22) to oil and coolant pressure</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -13107,7 +13131,7 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -13117,7 +13141,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SP-GNDOUT-B-ENG2</t>
+          <t>SP-GNDOUT-B-ENG3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -13128,7 +13152,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Sensor return splice - BH-B pin 29 (ECU B22) to oil and coolant pressure</t>
+          <t>Sensor return splice - BH-B pin 15 (ECU B22) to fuel pressure and gearbox speed</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -13138,7 +13162,7 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -13148,7 +13172,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SP-GNDOUT-B-ENG3</t>
+          <t>SP-GNDOUT-ENG</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -13159,17 +13183,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Sensor return splice - BH-B pin 15 (ECU B22) to fuel pressure and gearbox speed</t>
+          <t>Sensor return splice - BH-A pin 34 (ECU A24) to coolant temp, intake temp, throttle</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>solder splice</t>
+          <t>crimp splice</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -13179,7 +13203,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SP-GNDOUT-ENG</t>
+          <t>SP-GNDOUT-ENG2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
@@ -13190,17 +13214,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Sensor return splice - BH-A pin 34 (ECU A24) to coolant temp, intake temp, throttle</t>
+          <t>Sensor return splice - BH-A pin 18 (ECU A24) to MAP and flex sensor</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>crimp splice</t>
+          <t>solder splice</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -13210,7 +13234,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SP-GNDOUT-ENG2</t>
+          <t>SP-INJ-ENG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -13221,7 +13245,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Sensor return splice - BH-A pin 18 (ECU A24) to MAP and flex sensor</t>
+          <t>Injector +12 V splice - BH-A pin 2 (LOGIC INJ 15A) to injectors 1-4</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -13231,7 +13255,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -13241,7 +13265,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SP-INJ-ENG</t>
+          <t>SP-LAM12-B</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -13252,7 +13276,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Injector +12 V splice - BH-A pin 2 (LOGIC INJ 15A) to injectors 1-4</t>
+          <t>CAN-Lambda +12 V splice - 12 AWG from BH-B pin 95 to the 20 AWG lead</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -13262,7 +13286,7 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -13272,7 +13296,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SP-LAM12-B</t>
+          <t>SP-LAMG-B</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -13283,7 +13307,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>CAN-Lambda +12 V splice - 12 AWG from BH-B pin 95 to the 20 AWG lead</t>
+          <t>CAN-Lambda ground splice - 12 AWG from BH-B pin 96 to the 20 AWG lead</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -13303,7 +13327,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SP-LAMG-B</t>
+          <t>SP-SW12-ENG</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -13314,7 +13338,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CAN-Lambda ground splice - 12 AWG from BH-B pin 96 to the 20 AWG lead</t>
+          <t>Switched +12 V splice - BH-A pin 30 to boost solenoid and flex sensor</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -13324,7 +13348,7 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -13334,73 +13358,69 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SP-SW12-ENG</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
+          <t>R-TERM-END</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>120R 1/4W</t>
+        </is>
+      </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>splice</t>
+          <t>resistor</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Switched +12 V splice - BH-A pin 30 to boost solenoid and flex sensor</t>
+          <t>r_term_end</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>solder splice</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
       </c>
-      <c r="I45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>component lead 1 / 2 (as drawn)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>R-TERM-END</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>120R 1/4W</t>
-        </is>
-      </c>
+          <t>CAB-CAM</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>resistor</t>
+          <t>cable screen</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>r_term_end</t>
+          <t>cab_cam screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
       </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>component lead 1 / 2 (as drawn)</t>
-        </is>
-      </c>
+      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAB-CAM</t>
+          <t>CAB-CAN-LAM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
@@ -13411,7 +13431,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>cab_cam screen (floats at the device end)</t>
+          <t>cab_can_lam screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -13427,7 +13447,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAB-CAN-LAM</t>
+          <t>CAB-CRANK</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
@@ -13438,7 +13458,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>cab_can_lam screen (floats at the device end)</t>
+          <t>cab_crank screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -13454,7 +13474,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAB-CRANK</t>
+          <t>CAB-ETBM-AE</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -13465,7 +13485,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>cab_crank screen (floats at the device end)</t>
+          <t>cab_etbm_ae screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -13481,7 +13501,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAB-ETBM-AE</t>
+          <t>CAB-ETBS</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -13492,7 +13512,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>cab_etbm_ae screen (floats at the device end)</t>
+          <t>cab_etbs screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -13508,7 +13528,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAB-ETBS</t>
+          <t>CAB-FLEX</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -13519,7 +13539,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>cab_etbs screen (floats at the device end)</t>
+          <t>cab_flex screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -13535,7 +13555,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAB-FLEX</t>
+          <t>CAB-KNOCK1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -13546,7 +13566,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>cab_flex screen (floats at the device end)</t>
+          <t>cab_knock1 screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -13562,7 +13582,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAB-KNOCK1</t>
+          <t>CAB-TURBO</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -13573,7 +13593,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>cab_knock1 screen (floats at the device end)</t>
+          <t>cab_turbo screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -13589,7 +13609,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAB-TURBO</t>
+          <t>CAB-VSS</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -13600,7 +13620,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>cab_turbo screen (floats at the device end)</t>
+          <t>cab_vss screen (floats at the device end)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -13613,35 +13633,8 @@
       </c>
       <c r="I54" t="inlineStr"/>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>CAB-VSS</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>cable screen</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>cab_vss screen (floats at the device end)</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
+  <autoFilter ref="A1:I54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13874,12 +13867,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>w_eng_gnd</t>
+          <t>w_cop_gnd_e_ae</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Coil ground splice - ignition coils 1-4 to the engine block ground stud</t>
+          <t>Coil ground splice - ignition coils 1-4 to bulkhead pin 4 (POWER box NEG bar)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -13891,11 +13884,11 @@
         <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>8.550000000000001</v>
+        <v>6.6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>w_cop1g (18 AWG), w_cop2g (18 AWG), w_cop3g (18 AWG), w_cop4g (18 AWG), w_eng_gnd (10 AWG)</t>
+          <t>w_cop1g (18 AWG), w_cop2g (18 AWG), w_cop3g (18 AWG), w_cop4g (18 AWG), w_cop_gnd_e_ae (12 AWG)</t>
         </is>
       </c>
     </row>
@@ -14142,7 +14135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14269,7 +14262,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -14291,7 +14284,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -14313,7 +14306,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -14335,7 +14328,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -14357,12 +14350,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0413-214-1205</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -14379,7 +14372,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -14401,7 +14394,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -14423,7 +14416,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -14445,7 +14438,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -14467,7 +14460,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -14489,7 +14482,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>39</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -14511,7 +14504,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -14533,12 +14526,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>43</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>114019-ZZ</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -14555,12 +14548,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>114019-ZZ</t>
+          <t>114018-ZZ</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -14577,7 +14570,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -14599,12 +14592,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>114018-ZZ</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -14621,12 +14614,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>114018-ZZ</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -14643,7 +14636,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -14665,12 +14658,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>114018-ZZ</t>
+          <t>114019-ZZ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -14687,12 +14680,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>62</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>114019-ZZ</t>
+          <t>114017</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -14709,7 +14702,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>82</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -14731,7 +14724,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>86</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -14753,7 +14746,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>87</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -14775,7 +14768,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -14797,7 +14790,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>89</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -14819,7 +14812,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -14841,7 +14834,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>91</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -14863,7 +14856,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -14885,7 +14878,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -14907,7 +14900,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -14929,12 +14922,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>97</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>114017</t>
+          <t>0413-214-1205</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -14951,7 +14944,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>98</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -14973,7 +14966,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -14995,7 +14988,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -15017,7 +15010,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>101</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -15039,7 +15032,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>102</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -15053,30 +15046,8 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>DRB102-ENGINE</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>0413-214-1205</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>spare, sealing plug</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D42"/>
+  <autoFilter ref="A1:D41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15166,7 +15137,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wires: 98   Connectors / ends: 54   Splices: 13   Spare cavities: 41</t>
+          <t>Wires: 98   Connectors / ends: 53   Splices: 13   Spare cavities: 40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AB-engine: 6 in minimum breakout for a connector part-way along a line (Rev L)
Dan 2026-10-29: every connector sits at least 6 in (152 mm) off its main branch, unless it is the
last connector at the end of a run. The route-tree builder now gives such devices a 152 mm stub and
draws stub taps on the route line. Cam, coils 2-4 and CAN-Lambda lengths updated in the master;
DECISIONS B8, rev log, README harness.design notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -871,7 +871,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1005</t>
+          <t>1155</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>1052</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>795</t>
+          <t>947</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>618</t>
+          <t>749</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>618</t>
+          <t>749</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>618</t>
+          <t>749</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4779,7 +4779,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>618</t>
+          <t>749</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -6135,7 +6135,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>607</t>
+          <t>754</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>360</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>360</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>257</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>257</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>152</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -8195,7 +8195,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>152</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>607</t>
+          <t>754</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>607</t>
+          <t>754</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -11419,7 +11419,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>607</t>
+          <t>754</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>607</t>
+          <t>754</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">

</xml_diff>

<commit_message>
AB-engine: bulkhead 8 in above the trunk junction (+203 mm on bulkhead wires)
Dan 2026-10-29: the engine bulkhead sits 8 in (203 mm) above where the trunk meets the firewall.
route_trees gets root_drop_mm 203; build_drawings adds that segment at the root. Every AB-engine wire
with a bulkhead end is 203 mm longer (63 rows); no other wire changes. DECISIONS B8, Rev L note.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -651,7 +651,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1342</t>
+          <t>1545</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1088</t>
+          <t>1291</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1155</t>
+          <t>1358</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1052</t>
+          <t>1255</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>947</t>
+          <t>1150</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>1304</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>1304</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1023</t>
+          <t>1226</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1023</t>
+          <t>1226</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>852</t>
+          <t>1055</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>765</t>
+          <t>968</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>684</t>
+          <t>887</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>619</t>
+          <t>822</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>813</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>813</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1158</t>
+          <t>1361</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1158</t>
+          <t>1361</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>982</t>
+          <t>1185</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2615,7 +2615,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>982</t>
+          <t>1185</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1085</t>
+          <t>1288</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>827</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>827</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>827</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>827</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3307,7 +3307,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>827</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3423,7 +3423,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>827</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3535,7 +3535,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>827</t>
+          <t>1030</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1077</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>1077</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3883,7 +3883,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>1077</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3995,7 +3995,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>1077</t>
+          <t>1280</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>953</t>
+          <t>1156</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>1483</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1191</t>
+          <t>1394</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>952</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>952</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>952</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4779,7 +4779,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>952</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>1175</t>
+          <t>1378</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -5011,7 +5011,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>1175</t>
+          <t>1378</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>925</t>
+          <t>1128</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -5235,7 +5235,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>851</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>851</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5463,7 +5463,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>851</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>1007</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>1007</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -5807,7 +5807,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>1007</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>1251</t>
+          <t>1454</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>1251</t>
+          <t>1454</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -6135,7 +6135,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>957</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -10147,7 +10147,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>1175</t>
+          <t>1378</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>957</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>957</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -10515,7 +10515,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>795</t>
+          <t>998</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -10631,7 +10631,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>795</t>
+          <t>998</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -10747,7 +10747,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>704</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -10967,7 +10967,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>691</t>
+          <t>894</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>691</t>
+          <t>894</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -11191,7 +11191,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>867</t>
+          <t>1070</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -11303,7 +11303,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>577</t>
+          <t>780</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -11419,7 +11419,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>957</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>957</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>691</t>
+          <t>894</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">

</xml_diff>

<commit_message>
Knock sensor plug contacts: Bosch BDK 2.8 (was TBD)
Dan 2026-10-29 (A7): the Bosch Compact 1.1a housing 1 928 403 874 takes BDK 2.8 contacts with
individual wire seals (Bosch Compact 1.1a catalog). Parts table +2 BDK 2.8; drawings and BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -5260,7 +5260,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>BDK 2.8</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -5295,7 +5295,11 @@
       </c>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr"/>
-      <c r="Z43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>Knock plug contacts: Bosch BDK 2.8 with individual wire seals (Bosch Compact 1.1a catalog, 1 928 403 874; Dan 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5376,7 +5380,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>BDK 2.8</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -5411,7 +5415,11 @@
       </c>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="inlineStr"/>
-      <c r="Z44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>Knock plug contacts: Bosch BDK 2.8 with individual wire seals (Bosch Compact 1.1a catalog, 1 928 403 874; Dan 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -12590,7 +12598,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>BDK 2.8</t>
         </is>
       </c>
       <c r="G22" t="n">

</xml_diff>

<commit_message>
AB-engine parts: D-436-37 sensor-ground splice, DT cam plug, ETB motor cable
- SP-GNDOUT-ENG is a D-436-37 sealed crimp splice.
- Cam plug: DT06-3S-CE05 + W3S + 0462-201-16141 (sensor leads get the DT04-3P pair).
- ETB motor cable: 55A1821-18-2/0-9 (2-core 18 AWG Raychem).
- Parts table +2 rows; drawing set, wire lists and BOM regenerated.
- README: harness.design parts must stay in sync with the library (Dan 2026-10-29).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -3202,7 +3202,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>55A1821-18-2/0-9</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>55A1821-18-2/0-9</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>55A1821-18-2/0-9</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -4460,7 +4460,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>0462-201-16141</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -4495,7 +4495,11 @@
       </c>
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr"/>
-      <c r="Z36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4576,7 +4580,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>0462-201-16141</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -4611,7 +4615,11 @@
       </c>
       <c r="X37" t="inlineStr"/>
       <c r="Y37" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4692,7 +4700,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>0462-201-16141</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -4727,7 +4735,11 @@
       </c>
       <c r="X38" t="inlineStr"/>
       <c r="Y38" t="inlineStr"/>
-      <c r="Z38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -11833,7 +11845,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>DT06-3S-CE05</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -11846,10 +11858,14 @@
           <t>Cam Hall Sensor (RacerX)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>W3S</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>0462-201-16141</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -11860,7 +11876,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Deutsch DT / DTM cavity numbers (moulded on the housing)</t>
         </is>
       </c>
     </row>
@@ -13197,7 +13213,7 @@
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>crimp splice</t>
+          <t>D-436-37</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -13819,7 +13835,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>crimp splice</t>
+          <t>D-436-37</t>
         </is>
       </c>
       <c r="E5" t="n">

</xml_diff>

<commit_message>
Cam sensor leads are 20 AWG x 1 m (ZF GS1005-GS1007 datasheet); Needs Dan N68 closed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -4497,7 +4497,7 @@
       <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>Sensor: Cherry (ZF) GS1007 hall from the Racer X cam kit, bare leads brown +V / black signal / blue ground (Dan sensor sheet); lead gauge TBD. | Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
+          <t>Sensor: Cherry (ZF) GS1007 hall from the Racer X cam kit, bare leads brown +V / black signal / blue ground (Dan sensor sheet); leads 20 AWG x 1 m (ZF datasheet GS1005-GS1007, 2024-09-11), inside the DT pins' 16-20 AWG. | Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>Sensor: Cherry (ZF) GS1007 hall from the Racer X cam kit, bare leads brown +V / black signal / blue ground (Dan sensor sheet); lead gauge TBD. | Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
+          <t>Sensor: Cherry (ZF) GS1007 hall from the Racer X cam kit, bare leads brown +V / black signal / blue ground (Dan sensor sheet); leads 20 AWG x 1 m (ZF datasheet GS1005-GS1007, 2024-09-11), inside the DT pins' 16-20 AWG. | Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4737,7 @@
       <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>Sensor: Cherry (ZF) GS1007 hall from the Racer X cam kit, bare leads brown +V / black signal / blue ground (Dan sensor sheet); lead gauge TBD. | Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
+          <t>Sensor: Cherry (ZF) GS1007 hall from the Racer X cam kit, bare leads brown +V / black signal / blue ground (Dan sensor sheet); leads 20 AWG x 1 m (ZF datasheet GS1005-GS1007, 2024-09-11), inside the DT pins' 16-20 AWG. | Cam plug: harness side DT06-3S-CE05 + W3S + 0462-201-16141; the sensor's bare leads get DT04-3P + W3P + 0460-202-16141 (Dan 2026-10-29)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Starter S end is the Toyota 1-way plug 90980-11400 (Needs Dan N67, A)
- Master: STARTER-TRIGGER -> connector 90980-11400 pin 1 (RM1022E: 1-way, 4.8 mm tab, sealed), terminal from the
  Ballenger CONN-76058 kit (Sumitomo TS187 sealed female, 12-10 AWG); check the tab is 4.8 mm when fitting.
- Parts table +1 row; OPEN-ITEMS: N67 closed, Current state, History; drawings, wire lists, BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lug</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -668,7 +668,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Starter solenoid S (50) terminal post, spade</t>
+          <t>Starter solenoid S (50) terminal, 1-way plug</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -705,7 +705,7 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Starter solenoid S Candidate plug: Toyota 1-way sealed 90980-11400 (4.8 mm TS187 female; Toyota RM1022E housing list), sold for Toyota starters with a 12-10 AWG terminal; tab width to be checked at the car (Needs Dan N67). | Starter S crosses the firewall on its own DRB102 size-12 cavity (Dan 2026-10-27); 12 AWG: the DRB size-12 contact takes 12-14 AWG, solenoid S draw is brief, OEM lead is lighter</t>
+          <t>Starter solenoid S Plug 90980-11400 (Dan 2026-10-30, N67 A); kit Ballenger CONN-76058 has the 12-10 AWG terminal and seal; check the tab is 4.8 mm when fitting. | Starter S crosses the firewall on its own DRB102 size-12 cavity (Dan 2026-10-27); 12 AWG: the DRB size-12 contact takes 12-14 AWG, solenoid S draw is brief, OEM lead is lighter</t>
         </is>
       </c>
     </row>
@@ -12874,12 +12874,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TURBO-SPD</t>
+          <t>STARTER-TRIGGER</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DT06-3S-CE05</t>
+          <t>90980-11400</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -12889,40 +12889,36 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Turbo Speed Sensor</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>W3S</t>
-        </is>
-      </c>
+          <t>Starter solenoid S (50) terminal, 1-way plug</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0462-201-16141</t>
+          <t>in kit CONN-76058 (Sumitomo TS187 4.8 mm sealed female, 12-10 AWG)</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Deutsch DT / DTM cavity numbers (moulded on the housing)</t>
+          <t>single cavity (Toyota RM1022E housing list: 90980-11400 is 1-way, 4.8 mm tab, sealed)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>VSS</t>
+          <t>TURBO-SPD</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>90980-11143</t>
+          <t>DT06-3S-CE05</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -12932,13 +12928,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Gearbox VSS (Toyota 83181-20040, 3-wire) - actual road speed, plug 90980-11143</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
+          <t>Turbo Speed Sensor</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>W3S</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>0462-201-16141</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -12949,40 +12949,48 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Toyota 3-wire speed sensor pinout (wilbo666 wiki; Daniel 2026-09-28)</t>
+          <t>Deutsch DT / DTM cavity numbers (moulded on the housing)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>STARTER-TRIGGER</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>VSS</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>90980-11143</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>terminal</t>
+          <t>connector</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Starter solenoid S (50) terminal post, spade</t>
+          <t>Gearbox VSS (Toyota 83181-20040, 3-wire) - actual road speed, plug 90980-11143</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>8100-0461</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Toyota 3-wire speed sensor pinout (wilbo666 wiki; Daniel 2026-09-28)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">

</xml_diff>

<commit_message>
MR-S pump contacts (82998-12440 / -12500), coil contacts owned (PN TBD); Needs Dan N69-N70
- Master: MR-S middle / small plugs -> Toyota repair wire 82998-12440, big plug -> 82998-12500 (RM1022E;
  DIYElectricCar MR2 EHPS thread; both owned). Coil contacts owned with Dan's 90980-11885 plugs, maker PN unknown:
  8100-0461 (a guess) -> TBD (RM1022E: 2.3 II mm sealed). Coil pin-order note.
- BOM: coil and MR-S plugs counted as owned (never a buy). Parts table +2 rows.
- OPEN-ITEMS: Needs Dan N69 (82998-12500 lead gauge vs the 8 AWG pump feed), N70 (cavity counts), Current state, History.
- Drawings, wire lists and BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -780,7 +780,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -815,7 +815,11 @@
       </c>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -888,7 +892,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -923,7 +927,11 @@
       </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -996,7 +1004,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1031,7 +1039,11 @@
       </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1104,7 +1116,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1139,7 +1151,11 @@
       </c>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6296,7 +6312,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>82998-12440</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -6333,7 +6349,7 @@
       <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>EHPS enable +12 V | EHPS enable +12 V | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>EHPS enable +12 V | EHPS enable +12 V Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6424,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>82998-12440</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -6445,7 +6461,7 @@
       <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6536,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>82998-12440</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -6557,7 +6573,7 @@
       <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>
@@ -7435,7 +7451,7 @@
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -7477,7 +7493,7 @@
       <c r="Y62" t="inlineStr"/>
       <c r="Z62" t="inlineStr">
         <is>
-          <t>Coil 1 +12 V | Coil 1 +12 V</t>
+          <t>Coil 1 +12 V Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet. | Coil 1 +12 V</t>
         </is>
       </c>
     </row>
@@ -7551,7 +7567,7 @@
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -7591,7 +7607,11 @@
       </c>
       <c r="X63" t="inlineStr"/>
       <c r="Y63" t="inlineStr"/>
-      <c r="Z63" t="inlineStr"/>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7663,7 +7683,7 @@
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -7705,7 +7725,7 @@
       <c r="Y64" t="inlineStr"/>
       <c r="Z64" t="inlineStr">
         <is>
-          <t>Coil 2 +12 V | Coil 2 +12 V</t>
+          <t>Coil 2 +12 V Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet. | Coil 2 +12 V</t>
         </is>
       </c>
     </row>
@@ -7779,7 +7799,7 @@
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -7819,7 +7839,11 @@
       </c>
       <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr"/>
-      <c r="Z65" t="inlineStr"/>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7891,7 +7915,7 @@
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -7933,7 +7957,7 @@
       <c r="Y66" t="inlineStr"/>
       <c r="Z66" t="inlineStr">
         <is>
-          <t>Coil 3 +12 V | Coil 3 +12 V</t>
+          <t>Coil 3 +12 V Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet. | Coil 3 +12 V</t>
         </is>
       </c>
     </row>
@@ -8007,7 +8031,7 @@
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -8047,7 +8071,11 @@
       </c>
       <c r="X67" t="inlineStr"/>
       <c r="Y67" t="inlineStr"/>
-      <c r="Z67" t="inlineStr"/>
+      <c r="Z67" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8119,7 +8147,7 @@
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -8161,7 +8189,7 @@
       <c r="Y68" t="inlineStr"/>
       <c r="Z68" t="inlineStr">
         <is>
-          <t>Coil 4 +12 V | Coil 4 +12 V</t>
+          <t>Coil 4 +12 V Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet. | Coil 4 +12 V</t>
         </is>
       </c>
     </row>
@@ -8235,7 +8263,7 @@
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -8275,7 +8303,11 @@
       </c>
       <c r="X69" t="inlineStr"/>
       <c r="Y69" t="inlineStr"/>
-      <c r="Z69" t="inlineStr"/>
+      <c r="Z69" t="inlineStr">
+        <is>
+          <t>Contact owned with the plug (Dan 2026-10-30), maker PN not known; RM1022E: 90980-11885 takes 2.3 II mm sealed female contacts. Coil pins (1ZZ 90919-02239): 1 +B, 2 IGF, 3 IGT, 4 GND per an MS EFI forum note; the Racer X kit PDF lists the same pins right-to-left; no Toyota EWD in the repo yet.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -12033,7 +12065,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -12072,7 +12104,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -12111,7 +12143,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -12150,7 +12182,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8100-0461</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -12700,7 +12732,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>82998-12440</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -12739,7 +12771,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>82998-12440</t>
         </is>
       </c>
       <c r="G25" t="n">

</xml_diff>

<commit_message>
MR-S pump pins from the MR-S EWD (N70), spare cavities, N69 wire sizing
- Master: every MRS pin cites the MR-S EWD power steering page (P6 2-way, P7 8-way, P8 4-way);
  spare rows added for MRS-B 7 / 8 and MRS-C 3 / 4; wired pins already matched.
- OPEN-ITEMS: N70 closed; N69 now carries the load and derating (OEM 50 A EHPS fuse; 8 AWG right for the run).
- Drawings, wire lists, BOM regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -12743,7 +12743,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>MR-S (ZZW30) EWD power steering page (Dan 2026-10-30): P6 1 MH, 2 PGND; P7 1 IDUP, 2 SPD, 3 TC, 5 MRLY, 6 EFI, 7 TS; P8 1 IGB, 2 SIL, 4 WL</t>
         </is>
       </c>
     </row>
@@ -12782,7 +12782,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>MR-S (ZZW30) EWD power steering page (Dan 2026-10-30): P6 1 MH, 2 PGND; P7 1 IDUP, 2 SPD, 3 TC, 5 MRLY, 6 EFI, 7 TS; P8 1 IGB, 2 SIL, 4 WL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Step-down splices per B12: D-436-37 for the ETB 16 -> 20 AWG tails, hand solder + adhesive shrink for the EPS 8 AWG pigtail joins
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -3265,7 +3265,7 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>16 AWG core spliced to a short 20 AWG tail (M22759/16-20) at the ETB plug: the kit contact takes 24-20 AWG only (Dan 2026-10-30). | owner proposed: longer half (drawn today as w124_e on ECU-engine, 340 mm; w124_e_ae on ECU-engine, 590 mm)</t>
+          <t>16 AWG core joined to a short (&lt;= 150 mm) 20 AWG tail (M22759/16-20) at the ETB plug with a TE Raychem D-436-37 sealed crimp splice (20-16 AWG each side, 150 C): the kit contact takes 24-20 AWG only (Dan 2026-10-30). | owner proposed: longer half (drawn today as w124_e on ECU-engine, 340 mm; w124_e_ae on ECU-engine, 590 mm)</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3385,7 @@
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>16 AWG core spliced to a short 20 AWG tail (M22759/16-20) at the ETB plug: the kit contact takes 24-20 AWG only (Dan 2026-10-30). | owner proposed: longer half (drawn today as w215_e on ECU-engine, 340 mm; w215_e_ae on ECU-engine, 590 mm)</t>
+          <t>16 AWG core joined to a short (&lt;= 150 mm) 20 AWG tail (M22759/16-20) at the ETB plug with a TE Raychem D-436-37 sealed crimp splice (20-16 AWG each side, 150 C): the kit contact takes 24-20 AWG only (Dan 2026-10-30). | owner proposed: longer half (drawn today as w215_e on ECU-engine, 340 mm; w215_e_ae on ECU-engine, 590 mm)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Owned plugs from Dan's receipts: injector kits CONN-76270 (branches 18 AWG), crank plug 90980-10947, horn sockets 0462-209-1631
- Injectors: Ballenger CONN-76270 (black EV6/EV14, GT 150 20-16 AWG, seal 24-18 AWG), owned x4; +12 V branches 16 -> 18 AWG (B12 step 2)
- Crank: DT06-2S -> Toyota 90980-10947 (Ballenger CONN-75800, owned), mates the sensor's own socket; pin order TBD
- Horn sockets: owned gold 0462-209-1631 (Dan, 2a)
- Needs Dan N80 (ETB housing number), N81 (EPS pigtail AWG), N82 (GXL/TXL use)
- harness.design lDDj + library 5LO8 synced; drawings and BOM regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -1664,7 +1664,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>0462-201-16141</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -5675,7 +5675,11 @@
       </c>
       <c r="X46" t="inlineStr"/>
       <c r="Y46" t="inlineStr"/>
-      <c r="Z46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Crank plug: Toyota 90980-10947 (Sumitomo 2-way TS, Ballenger kit CONN-75800, owned; Dan 2026-10-31) mates the sensor's own socket; which cavity is signal vs ground is TBD (EWD)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5756,7 +5760,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>0462-201-16141</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -5791,7 +5795,11 @@
       </c>
       <c r="X47" t="inlineStr"/>
       <c r="Y47" t="inlineStr"/>
-      <c r="Z47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>Crank plug: Toyota 90980-10947 (Sumitomo 2-way TS, Ballenger kit CONN-75800, owned; Dan 2026-10-31) mates the sensor's own socket; which cavity is signal vs ground is TBD (EWD)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9062,7 +9070,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -9072,14 +9080,14 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -9121,7 +9129,7 @@
       <c r="Y76" t="inlineStr"/>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>Injector 1 +12 V | Injector 1 +12 V</t>
+          <t>Injector 1 +12 V | Injector 1 +12 V | Injector plugs: Ballenger CONN-76270 kits (black EV6/EV14 housing, GT 150 female 20-16 AWG, white cable seal 24-18 AWG), owned x4 (Dan 2026-10-31). Branches 18 AWG because the seal stops at 18 AWG (B12 step 2); load ~1.2 A each, INJ fuse 7.5 A.</t>
         </is>
       </c>
     </row>
@@ -9178,7 +9186,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -9188,14 +9196,14 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -9294,7 +9302,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -9304,14 +9312,14 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9410,7 +9418,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -9420,14 +9428,14 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -12205,7 +12213,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DT06-2S-CE05</t>
+          <t>90980-10947</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -12218,14 +12226,10 @@
           <t>Crank VR Sensor (36-2)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>W2S</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0462-201-16141</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -12236,7 +12240,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Deutsch DT / DTM cavity numbers (moulded on the housing)</t>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -12482,7 +12486,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -12498,7 +12502,7 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -12521,7 +12525,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -12537,7 +12541,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -12560,7 +12564,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12576,7 +12580,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -12599,7 +12603,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -12615,7 +12619,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -13791,11 +13795,11 @@
         <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>7.32</v>
+        <v>5.37</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>w_inj_pwr_e_ae (14 AWG), w211 (16 AWG), w212 (16 AWG), w213 (16 AWG), w214 (16 AWG)</t>
+          <t>w_inj_pwr_e_ae (14 AWG), w211 (18 AWG), w212 (18 AWG), w213 (18 AWG), w214 (18 AWG)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Owned plugs from Dan's receipts: injector kits CONN-76270 (branches 18 AWG), crank plug 90980-10947, horn sockets 0462-209-1631 (#428)
- Injectors: Ballenger CONN-76270 (black EV6/EV14, GT 150 20-16 AWG, seal 24-18 AWG), owned x4; +12 V branches 16 -> 18 AWG (B12 step 2)
- Crank: DT06-2S -> Toyota 90980-10947 (Ballenger CONN-75800, owned), mates the sensor's own socket; pin order TBD
- Horn sockets: owned gold 0462-209-1631 (Dan, 2a)
- Needs Dan N80 (ETB housing number), N81 (EPS pigtail AWG), N82 (GXL/TXL use)
- harness.design lDDj + library 5LO8 synced; drawings and BOM regenerated


Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -1664,7 +1664,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>0462-201-16141</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -5675,7 +5675,11 @@
       </c>
       <c r="X46" t="inlineStr"/>
       <c r="Y46" t="inlineStr"/>
-      <c r="Z46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>Crank plug: Toyota 90980-10947 (Sumitomo 2-way TS, Ballenger kit CONN-75800, owned; Dan 2026-10-31) mates the sensor's own socket; which cavity is signal vs ground is TBD (EWD)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5756,7 +5760,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>0462-201-16141</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -5791,7 +5795,11 @@
       </c>
       <c r="X47" t="inlineStr"/>
       <c r="Y47" t="inlineStr"/>
-      <c r="Z47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>Crank plug: Toyota 90980-10947 (Sumitomo 2-way TS, Ballenger kit CONN-75800, owned; Dan 2026-10-31) mates the sensor's own socket; which cavity is signal vs ground is TBD (EWD)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9062,7 +9070,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -9072,14 +9080,14 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N76" t="inlineStr"/>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -9121,7 +9129,7 @@
       <c r="Y76" t="inlineStr"/>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>Injector 1 +12 V | Injector 1 +12 V</t>
+          <t>Injector 1 +12 V | Injector 1 +12 V | Injector plugs: Ballenger CONN-76270 kits (black EV6/EV14 housing, GT 150 female 20-16 AWG, white cable seal 24-18 AWG), owned x4 (Dan 2026-10-31). Branches 18 AWG because the seal stops at 18 AWG (B12 step 2); load ~1.2 A each, INJ fuse 7.5 A.</t>
         </is>
       </c>
     </row>
@@ -9178,7 +9186,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -9188,14 +9196,14 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N77" t="inlineStr"/>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -9294,7 +9302,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -9304,14 +9312,14 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9410,7 +9418,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -9420,14 +9428,14 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>M22759/16-16-2</t>
+          <t>M22759/16-18-2</t>
         </is>
       </c>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
         <is>
-          <t>12191819</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -12205,7 +12213,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DT06-2S-CE05</t>
+          <t>90980-10947</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -12218,14 +12226,10 @@
           <t>Crank VR Sensor (36-2)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>W2S</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0462-201-16141</t>
+          <t>in kit CONN-75800</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -12236,7 +12240,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Deutsch DT / DTM cavity numbers (moulded on the housing)</t>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -12482,7 +12486,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -12498,7 +12502,7 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -12521,7 +12525,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -12537,7 +12541,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -12560,7 +12564,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12576,7 +12580,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -12599,7 +12603,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>15419715</t>
+          <t>CONN-76270</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -12615,7 +12619,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>12191819, 15326426</t>
+          <t>in kit CONN-76270</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -13791,11 +13795,11 @@
         <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>7.32</v>
+        <v>5.37</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>w_inj_pwr_e_ae (14 AWG), w211 (16 AWG), w212 (16 AWG), w213 (16 AWG), w214 (16 AWG)</t>
+          <t>w_inj_pwr_e_ae (14 AWG), w211 (18 AWG), w212 (18 AWG), w213 (18 AWG), w214 (18 AWG)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETB 18 AWG contact approved (TE C-967616) and EPS pigtail sizes from Toyota RM06H0E (N80, N81)
- ETB: 5-965906-1 (0.5-0.75 mm2, 20-18 AWG) + seal 1-967067-1 are on TE drawing C-967616 for housing 1-967616-1
- EPS: 82998-12500 lead is 8 mm2 (matches the 8 AWG run); 82998-12440 lead is 2.0 mm2
- DECISIONS B12 cases, tracker, drawings regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -3265,7 +3265,7 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (20-18 AWG, 7.5 A) in place of the kit contact (24-20 AWG); TEST-FIT in the Bosch housing before building - no Bosch fit approval found. Fallback if it fails: 20 AWG whole circuit (kit contact, 55A1821-20 cable), ETB fuse 5 A. Motor ~2 A typical, &lt; 10 A max (Bosch data sheet). | owner proposed: longer half (drawn today as w124_e on ECU-engine, 340 mm; w124_e_ae on ECU-engine, 590 mm)</t>
+          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (0.5-0.75 mm2, 20-18 AWG, 7.5 A) with green seal 1-967067-1 (insulation 1.4-2.1 mm): both on TE drawing C-967616 for housing 1-967616-1 (the Bosch 6-pin MQS plug); crimp pull-test one, 18 AWG is the top of the range. Motor ~2 A typical, &lt; 10 A max (Bosch data sheet). | owner proposed: longer half (drawn today as w124_e on ECU-engine, 340 mm; w124_e_ae on ECU-engine, 590 mm)</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3385,7 @@
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (20-18 AWG, 7.5 A) in place of the kit contact (24-20 AWG); TEST-FIT in the Bosch housing before building - no Bosch fit approval found. Fallback if it fails: 20 AWG whole circuit (kit contact, 55A1821-20 cable), ETB fuse 5 A. | owner proposed: longer half (drawn today as w215_e on ECU-engine, 340 mm; w215_e_ae on ECU-engine, 590 mm)</t>
+          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (0.5-0.75 mm2, 20-18 AWG, 7.5 A) with green seal 1-967067-1 (insulation 1.4-2.1 mm): both on TE drawing C-967616 for housing 1-967616-1 (the Bosch 6-pin MQS plug); crimp pull-test one, 18 AWG is the top of the range. | owner proposed: longer half (drawn today as w215_e on ECU-engine, 340 mm; w215_e_ae on ECU-engine, 590 mm)</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>EHPS enable +12 V | EHPS enable +12 V Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>EHPS enable +12 V | EHPS enable +12 V Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); lead 2.0 mm2 (about 14 AWG, Toyota RM06H0E section F), larger than the harness wire, which solder-splices to it. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>
@@ -6469,7 +6469,7 @@
       <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); lead 2.0 mm2 (about 14 AWG, Toyota RM06H0E section F), larger than the harness wire, which solder-splices to it. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>
@@ -6581,7 +6581,7 @@
       <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); lead 2.0 mm2 (about 14 AWG, Toyota RM06H0E section F), larger than the harness wire, which solder-splices to it. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ETB 18 AWG contact approved (TE C-967616) and EPS pigtail sizes from Toyota RM06H0E (N80, N81) (#430)
- ETB: 5-965906-1 (0.5-0.75 mm2, 20-18 AWG) + seal 1-967067-1 are on TE drawing C-967616 for housing 1-967616-1
- EPS: 82998-12500 lead is 8 mm2 (matches the 8 AWG run); 82998-12440 lead is 2.0 mm2
- DECISIONS B12 cases, tracker, drawings regenerated


Claude-Session: https://claude.ai/code/session_01CSUgSkGzAUx8321hYpGMbx

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -3265,7 +3265,7 @@
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (20-18 AWG, 7.5 A) in place of the kit contact (24-20 AWG); TEST-FIT in the Bosch housing before building - no Bosch fit approval found. Fallback if it fails: 20 AWG whole circuit (kit contact, 55A1821-20 cable), ETB fuse 5 A. Motor ~2 A typical, &lt; 10 A max (Bosch data sheet). | owner proposed: longer half (drawn today as w124_e on ECU-engine, 340 mm; w124_e_ae on ECU-engine, 590 mm)</t>
+          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (0.5-0.75 mm2, 20-18 AWG, 7.5 A) with green seal 1-967067-1 (insulation 1.4-2.1 mm): both on TE drawing C-967616 for housing 1-967616-1 (the Bosch 6-pin MQS plug); crimp pull-test one, 18 AWG is the top of the range. Motor ~2 A typical, &lt; 10 A max (Bosch data sheet). | owner proposed: longer half (drawn today as w124_e on ECU-engine, 340 mm; w124_e_ae on ECU-engine, 590 mm)</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3385,7 @@
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (20-18 AWG, 7.5 A) in place of the kit contact (24-20 AWG); TEST-FIT in the Bosch housing before building - no Bosch fit approval found. Fallback if it fails: 20 AWG whole circuit (kit contact, 55A1821-20 cable), ETB fuse 5 A. | owner proposed: longer half (drawn today as w215_e on ECU-engine, 340 mm; w215_e_ae on ECU-engine, 590 mm)</t>
+          <t>18 AWG the whole circuit, no tail (Dan 2026-10-30, N77 A): TE MQS 0.63 sealed contact 5-965906-1 (0.5-0.75 mm2, 20-18 AWG, 7.5 A) with green seal 1-967067-1 (insulation 1.4-2.1 mm): both on TE drawing C-967616 for housing 1-967616-1 (the Bosch 6-pin MQS plug); crimp pull-test one, 18 AWG is the top of the range. | owner proposed: longer half (drawn today as w215_e on ECU-engine, 340 mm; w215_e_ae on ECU-engine, 590 mm)</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr">
         <is>
-          <t>EHPS enable +12 V | EHPS enable +12 V Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>EHPS enable +12 V | EHPS enable +12 V Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); lead 2.0 mm2 (about 14 AWG, Toyota RM06H0E section F), larger than the harness wire, which solder-splices to it. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>
@@ -6469,7 +6469,7 @@
       <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr">
         <is>
-          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); lead 2.0 mm2 (about 14 AWG, Toyota RM06H0E section F), larger than the harness wire, which solder-splices to it. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>
@@ -6581,7 +6581,7 @@
       <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr">
         <is>
-          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); the harness wire splices to its lead. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
+          <t>Contact: Toyota repair wire 82998-12440 (2.3 II mm sealed female + seal + about 6 in lead, owned; Toyota RM1022E lists it for 90980-10897 / -10942; DIYElectricCar MR2 EHPS thread); lead 2.0 mm2 (about 14 AWG, Toyota RM06H0E section F), larger than the harness wire, which solder-splices to it. | ECU engine harness owns it: leaves the bulkhead in the engine loom to the MR-S pump plug (Dan 2026-10-29); harness C keeps the 8 AWG pump power and ground</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gearbox speed sensor on ECU +8V, pull-up off; row 169 closed (Dan 2026-11-01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014aA8s41WDmzkdeUSzti3t8
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -4676,7 +4676,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>w_vss_12v</t>
+          <t>w_vss_8v</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
+          <t>+8 V to gearbox speed sensor</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>8V</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -4772,19 +4772,19 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>8V</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>ST185-AB-cabin w_rail_sw12_b_c_ac at DRB102-CABIN 67, to splice SP-SW12</t>
+          <t>ST185-AB-cabin w_rail_sp_8v_vss_c at DRB102-CABIN 67, to splice SP-8V</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>+12 V gearbox speed | +12 V gearbox speed</t>
+          <t>Dan 2026-11-01: VSS on ECU +8V; core colour set by cable CAB-VSS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gearbox speed sensor on ECU +8V, pull-up off; row 169 closed (Dan 2026-11-01) (#460)
Claude-Session: https://claude.ai/code/session_014aA8s41WDmzkdeUSzti3t8

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
+++ b/docs/harness/wirelists/ST185-AB-engine-wirelist.xlsx
@@ -4676,7 +4676,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>w_vss_12v</t>
+          <t>w_vss_8v</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>EFI relay k_efi -&gt; LOGIC SW12 5 A fuse</t>
+          <t>+8 V to gearbox speed sensor</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>8V</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -4772,19 +4772,19 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>SW12</t>
+          <t>8V</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>ST185-AB-cabin w_rail_sw12_b_c_ac at DRB102-CABIN 67, to splice SP-SW12</t>
+          <t>ST185-AB-cabin w_rail_sp_8v_vss_c at DRB102-CABIN 67, to splice SP-8V</t>
         </is>
       </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>+12 V gearbox speed | +12 V gearbox speed</t>
+          <t>Dan 2026-11-01: VSS on ECU +8V; core colour set by cable CAB-VSS</t>
         </is>
       </c>
     </row>

</xml_diff>